<commit_message>
Portsmouth (RHU): drop stale alt press address, re-verify primary
pho-tr.communications@nhs.net confirmed against the trust's own
contact-us page on 2026-08-18. Removed the superseded alt
communications@porthosp.nhs.uk, which was reported as wrong.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/trust-contacts.xlsx
+++ b/trust-contacts.xlsx
@@ -5342,11 +5342,7 @@
           <t>pho-tr.communications@nhs.net</t>
         </is>
       </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>communications@porthosp.nhs.uk</t>
-        </is>
-      </c>
+      <c r="D126" t="inlineStr"/>
       <c r="E126" t="inlineStr">
         <is>
           <t>https://www.porthosp.nhs.uk/about-us/contact-us</t>
@@ -5369,7 +5365,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>in progress</t>
+          <t>2026-08-18: press_email pho-tr.communications@nhs.net re-verified against the trust's own contact-us page. Stale alt communications@porthosp.nhs.uk removed - reported as wrong. Note: Isle of Wight NHS Trust (R1F) legitimately shares this same comms inbox.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verify 4 trusts left mid-sweep; repoint dead Wye Valley FOI URL
RHW, RL1, RL4 and RLQ carried a leftover 'in progress' note from an
interrupted refresh batch. All eight press/FOI addresses re-verified
against the trusts' own pages on 2026-08-18 and all were correct.

Wye Valley's stored foi_source_url now 404s; repointed to the live
make-a-freedom-of-information-request.aspx page. Address unchanged.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/trust-contacts.xlsx
+++ b/trust-contacts.xlsx
@@ -5478,7 +5478,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>in progress</t>
+          <t>2026-08-18: press and FOI emails both re-verified against the trust's own contact-us page.</t>
         </is>
       </c>
     </row>
@@ -7195,7 +7195,7 @@
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>in progress</t>
+          <t>2026-08-18: press and FOI emails both re-verified against the trust's own pages. Trust asks media to route all enquiries via the press office rather than contacting staff directly.</t>
         </is>
       </c>
     </row>
@@ -7339,7 +7339,7 @@
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>in progress</t>
+          <t>2026-08-18: press and FOI emails both re-verified against the trust's own contact-us page. Press address is listed there as 'Website Enquiries / Media / Press', so it is not media-only.</t>
         </is>
       </c>
     </row>
@@ -8442,12 +8442,12 @@
       <c r="G204" t="inlineStr"/>
       <c r="H204" t="inlineStr">
         <is>
-          <t>https://www.wyevalley.nhs.uk/about-us/information-requests/freedom-of-information-requests.aspx</t>
+          <t>https://www.wyevalley.nhs.uk/about-us/information-requests/make-a-freedom-of-information-request.aspx</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>in progress</t>
+          <t>2026-08-18: press and FOI emails both re-verified against the trust's own pages. foi_source_url repointed - the old freedom-of-information-requests.aspx now 404s. Press office page also lists three named comms staff (John Burnett, comms and engagement manager; Amanda Millichip and Fiona Gurney, comms officers) on 01432 372928.</t>
         </is>
       </c>
     </row>

</xml_diff>